<commit_message>
Pushed using deploy.sh script
</commit_message>
<xml_diff>
--- a/backend/cards.xlsx
+++ b/backend/cards.xlsx
@@ -507,7 +507,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>আমদর-বষয</t>
+          <t>school-history</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>যগযগর-ঠকন</t>
+          <t>contact-address</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>আমদর-ছতর-ছতর</t>
+          <t>number-of-students-studying</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>অধযযনরত-শকষরথর-সখয</t>
+          <t>our-faculty</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>নটশ</t>
+          <t>notices</t>
         </is>
       </c>
       <c r="J17" t="n">

</xml_diff>